<commit_message>
updating with dec 25 and cleaning for running totals
</commit_message>
<xml_diff>
--- a/ETO_Fluoro_Use.xlsx
+++ b/ETO_Fluoro_Use.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11003"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD2B583A-D15B-9643-8338-8BC66FC9F21B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8DDCF99-1793-614C-AD92-3007814B86B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ETO Use" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="106">
   <si>
     <t>Date</t>
   </si>
@@ -343,6 +343,12 @@
   </si>
   <si>
     <t>01-01777-5000-54903702-64303</t>
+  </si>
+  <si>
+    <t>CL015, CL017</t>
+  </si>
+  <si>
+    <t>CL017</t>
   </si>
 </sst>
 </file>
@@ -1891,7 +1897,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="27.6640625" bestFit="1" customWidth="1"/>
@@ -2285,6 +2291,23 @@
         <v>53</v>
       </c>
     </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>105</v>
+      </c>
+      <c r="B20">
+        <v>39143</v>
+      </c>
+      <c r="C20" t="s">
+        <v>32</v>
+      </c>
+      <c r="D20" t="s">
+        <v>13</v>
+      </c>
+      <c r="E20" t="s">
+        <v>54</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2294,7 +2317,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:C60"/>
+  <dimension ref="A1:C64"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="29.1640625" bestFit="1" customWidth="1"/>
@@ -2782,6 +2805,38 @@
         <v>79</v>
       </c>
     </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A61" s="1">
+        <v>45996</v>
+      </c>
+      <c r="B61" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A62" s="1">
+        <v>45999</v>
+      </c>
+      <c r="B62" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A63" s="1">
+        <v>46003</v>
+      </c>
+      <c r="B63" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A64" s="1">
+        <v>46013</v>
+      </c>
+      <c r="B64" t="s">
+        <v>104</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -2790,7 +2845,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D46EC14E-6917-0943-8C04-E0E228EF2377}">
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -2945,6 +3000,46 @@
         <v>19</v>
       </c>
     </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A20" s="1">
+        <v>45992</v>
+      </c>
+      <c r="B20" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A21" s="1">
+        <v>45992</v>
+      </c>
+      <c r="B21" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22" s="1">
+        <v>45999</v>
+      </c>
+      <c r="B22" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23" s="1">
+        <v>46001</v>
+      </c>
+      <c r="B23" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A24" s="1">
+        <v>46007</v>
+      </c>
+      <c r="B24" t="s">
+        <v>19</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
updates through march 26
</commit_message>
<xml_diff>
--- a/ETO_Fluoro_Use.xlsx
+++ b/ETO_Fluoro_Use.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11003"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10201"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8DDCF99-1793-614C-AD92-3007814B86B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5D7932F-7E62-BB48-8102-8FE28FB75386}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="31920" yWindow="1300" windowWidth="30240" windowHeight="18880" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ETO Use" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="106">
   <si>
     <t>Date</t>
   </si>
@@ -2317,7 +2317,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:C64"/>
+  <dimension ref="A1:C71"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="29.1640625" bestFit="1" customWidth="1"/>
@@ -2837,6 +2837,62 @@
         <v>104</v>
       </c>
     </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A65" s="1">
+        <v>46037</v>
+      </c>
+      <c r="B65" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A66" s="1">
+        <v>46052</v>
+      </c>
+      <c r="B66" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A67" s="1">
+        <v>46063</v>
+      </c>
+      <c r="B67" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A68" s="1">
+        <v>46069</v>
+      </c>
+      <c r="B68" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A69" s="1">
+        <v>46077</v>
+      </c>
+      <c r="B69" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A70" s="1">
+        <v>46088</v>
+      </c>
+      <c r="B70" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A71" s="1">
+        <v>46098</v>
+      </c>
+      <c r="B71" t="s">
+        <v>79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -2845,7 +2901,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D46EC14E-6917-0943-8C04-E0E228EF2377}">
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -3040,6 +3096,22 @@
         <v>19</v>
       </c>
     </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A25" s="1">
+        <v>46086</v>
+      </c>
+      <c r="B25" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A26" s="1">
+        <v>46097</v>
+      </c>
+      <c r="B26" t="s">
+        <v>47</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
updating to add PM001"
</commit_message>
<xml_diff>
--- a/ETO_Fluoro_Use.xlsx
+++ b/ETO_Fluoro_Use.xlsx
@@ -1,17 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10621"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F299FA85-9FF9-D348-966F-142E45316AF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72B44019-D0F4-FD43-846D-768717AE6E6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31920" yWindow="1300" windowWidth="30240" windowHeight="18880" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ETO Use" sheetId="1" r:id="rId1"/>
     <sheet name="CL Codes" sheetId="2" r:id="rId2"/>
     <sheet name="eto_use_alt" sheetId="3" r:id="rId3"/>
     <sheet name="fluoro_use" sheetId="4" r:id="rId4"/>
+    <sheet name="PM Cost" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -31,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="114">
   <si>
     <t>Date</t>
   </si>
@@ -355,13 +356,34 @@
   </si>
   <si>
     <t>Ranjan/DiBella</t>
+  </si>
+  <si>
+    <t>CL019</t>
+  </si>
+  <si>
+    <t>01-01777-2000-30203-64303-1</t>
+  </si>
+  <si>
+    <t>ECMO Training</t>
+  </si>
+  <si>
+    <t>PM000</t>
+  </si>
+  <si>
+    <t>Account to cover PM balance</t>
+  </si>
+  <si>
+    <t>Cost</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
+  </numFmts>
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -416,6 +438,12 @@
       <name val="Aptos"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Century Gothic"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -443,7 +471,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -474,6 +502,8 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1903,7 +1933,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="27.6640625" bestFit="1" customWidth="1"/>
@@ -1955,27 +1985,21 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>51</v>
-      </c>
-      <c r="C3" t="s">
-        <v>27</v>
+        <v>111</v>
       </c>
       <c r="D3" t="s">
-        <v>4</v>
+        <v>53</v>
       </c>
       <c r="E3" t="s">
         <v>53</v>
       </c>
       <c r="F3" t="s">
-        <v>35</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>88</v>
+        <v>51</v>
       </c>
       <c r="C4" t="s">
         <v>27</v>
@@ -1989,134 +2013,134 @@
       <c r="F4" t="s">
         <v>35</v>
       </c>
-      <c r="G4">
-        <v>2148</v>
-      </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>89</v>
+        <v>16</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>88</v>
       </c>
       <c r="C5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D5" t="s">
-        <v>46</v>
+        <v>4</v>
       </c>
       <c r="E5" t="s">
         <v>53</v>
       </c>
       <c r="F5" t="s">
-        <v>36</v>
+        <v>35</v>
+      </c>
+      <c r="G5">
+        <v>2148</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>90</v>
+        <v>18</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>89</v>
       </c>
       <c r="C6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D6" t="s">
-        <v>11</v>
+        <v>46</v>
       </c>
       <c r="E6" t="s">
         <v>53</v>
       </c>
       <c r="F6" t="s">
-        <v>37</v>
-      </c>
-      <c r="G6">
-        <v>2140</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>20</v>
-      </c>
-      <c r="B7" s="6"/>
+        <v>19</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>90</v>
+      </c>
       <c r="C7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D7" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="E7" t="s">
         <v>53</v>
       </c>
+      <c r="F7" t="s">
+        <v>37</v>
+      </c>
+      <c r="G7">
+        <v>2140</v>
+      </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>21</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>91</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="B8" s="6"/>
       <c r="C8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D8" t="s">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="E8" t="s">
-        <v>54</v>
-      </c>
-      <c r="F8" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>22</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>92</v>
+        <v>21</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>91</v>
       </c>
       <c r="C9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D9" t="s">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="E9" t="s">
         <v>54</v>
       </c>
       <c r="F9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>23</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>93</v>
+        <v>22</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>92</v>
       </c>
       <c r="C10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D10" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E10" t="s">
         <v>54</v>
       </c>
       <c r="F10" t="s">
-        <v>84</v>
+        <v>39</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>24</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>94</v>
+        <v>23</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>93</v>
       </c>
       <c r="C11" t="s">
         <v>33</v>
@@ -2128,80 +2152,77 @@
         <v>54</v>
       </c>
       <c r="F11" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>25</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>95</v>
+        <v>24</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>94</v>
       </c>
       <c r="C12" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D12" t="s">
-        <v>44</v>
+        <v>8</v>
       </c>
       <c r="E12" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F12" t="s">
-        <v>40</v>
+        <v>85</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>26</v>
-      </c>
-      <c r="B13" s="8" t="s">
-        <v>96</v>
+        <v>25</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>95</v>
       </c>
       <c r="C13" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D13" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
       <c r="E13" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F13" t="s">
-        <v>41</v>
-      </c>
-      <c r="G13">
-        <v>2200</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>57</v>
-      </c>
-      <c r="B14" s="9" t="s">
-        <v>97</v>
+        <v>26</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>96</v>
       </c>
       <c r="C14" t="s">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="D14" t="s">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="E14" t="s">
         <v>53</v>
       </c>
       <c r="F14" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="G14">
-        <v>1848</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>58</v>
-      </c>
-      <c r="B15" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="B15" s="9" t="s">
         <v>97</v>
       </c>
       <c r="C15" t="s">
@@ -2214,84 +2235,90 @@
         <v>53</v>
       </c>
       <c r="F15" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G15">
-        <v>2057</v>
+        <v>1848</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>56</v>
-      </c>
-      <c r="B16" s="10" t="s">
-        <v>98</v>
+        <v>58</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>97</v>
       </c>
       <c r="C16" t="s">
-        <v>27</v>
+        <v>59</v>
       </c>
       <c r="D16" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E16" t="s">
         <v>53</v>
       </c>
       <c r="F16" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G16">
-        <v>2336</v>
+        <v>2057</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>76</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>99</v>
+        <v>56</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>98</v>
       </c>
       <c r="C17" t="s">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="D17" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E17" t="s">
         <v>53</v>
       </c>
+      <c r="F17" t="s">
+        <v>62</v>
+      </c>
       <c r="G17">
-        <v>2348</v>
+        <v>2336</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>79</v>
-      </c>
-      <c r="B18" s="11" t="s">
-        <v>100</v>
+        <v>76</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>99</v>
       </c>
       <c r="C18" t="s">
-        <v>81</v>
+        <v>59</v>
       </c>
       <c r="D18" t="s">
-        <v>82</v>
+        <v>5</v>
       </c>
       <c r="E18" t="s">
         <v>53</v>
       </c>
+      <c r="G18">
+        <v>2348</v>
+      </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>102</v>
-      </c>
-      <c r="B19" t="s">
-        <v>103</v>
+        <v>79</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>100</v>
       </c>
       <c r="C19" t="s">
-        <v>59</v>
+        <v>81</v>
       </c>
       <c r="D19" t="s">
-        <v>5</v>
+        <v>82</v>
       </c>
       <c r="E19" t="s">
         <v>53</v>
@@ -2299,33 +2326,73 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>105</v>
-      </c>
-      <c r="B20">
-        <v>39143</v>
+        <v>102</v>
+      </c>
+      <c r="B20" t="s">
+        <v>103</v>
       </c>
       <c r="C20" t="s">
-        <v>32</v>
+        <v>59</v>
       </c>
       <c r="D20" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="E20" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
+        <v>105</v>
+      </c>
+      <c r="B21">
+        <v>39143</v>
+      </c>
+      <c r="C21" t="s">
+        <v>32</v>
+      </c>
+      <c r="D21" t="s">
+        <v>13</v>
+      </c>
+      <c r="E21" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
         <v>106</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C22" t="s">
         <v>34</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D22" t="s">
         <v>107</v>
       </c>
-      <c r="E21" t="s">
+      <c r="E22" t="s">
         <v>55</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>108</v>
+      </c>
+      <c r="B23" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="C23" t="s">
+        <v>27</v>
+      </c>
+      <c r="D23" t="s">
+        <v>4</v>
+      </c>
+      <c r="E23" t="s">
+        <v>53</v>
+      </c>
+      <c r="F23" t="s">
+        <v>110</v>
+      </c>
+      <c r="G23">
+        <v>1813</v>
       </c>
     </row>
   </sheetData>
@@ -2337,7 +2404,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:C72"/>
+  <dimension ref="A1:C80"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="29.1640625" bestFit="1" customWidth="1"/>
@@ -2921,6 +2988,70 @@
         <v>106</v>
       </c>
     </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A73" s="1">
+        <v>46149</v>
+      </c>
+      <c r="B73" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A74" s="1">
+        <v>46150</v>
+      </c>
+      <c r="B74" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A75" s="1">
+        <v>46170</v>
+      </c>
+      <c r="B75" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A76" s="1">
+        <v>46175</v>
+      </c>
+      <c r="B76" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A77" s="1">
+        <v>46177</v>
+      </c>
+      <c r="B77" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A78" s="1">
+        <v>46185</v>
+      </c>
+      <c r="B78" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A79" s="1">
+        <v>46191</v>
+      </c>
+      <c r="B79" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A80" s="1">
+        <v>46196</v>
+      </c>
+      <c r="B80" t="s">
+        <v>106</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -2929,7 +3060,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D46EC14E-6917-0943-8C04-E0E228EF2377}">
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -3140,8 +3271,48 @@
         <v>47</v>
       </c>
     </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A27" s="1">
+        <v>46203</v>
+      </c>
+      <c r="B27" t="s">
+        <v>76</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A1E41A3-E161-2249-B775-009343A1E366}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" s="1">
+        <v>46204</v>
+      </c>
+      <c r="B2" s="13">
+        <v>2500</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{170051ed-867f-4092-a6af-8a42e27b7e09}" enabled="1" method="Standard" siteId="{5217e0e7-539d-4563-b1bf-7c6dcf074f91}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>